<commit_message>
align oatside pricing with run-date diesel rules
Switch Oatside billing to configurable fuel-linked pricing by daily run date so April/May base-rate policy and floor rules can be audited and adjusted without code changes, while enforcing 50% return-job charging consistently.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
+++ b/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Info" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Customer_Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Customer_Trips_Per_Day" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Audit_Log" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Trip_Detail" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Trips_Pricing_All" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Unmatched_Log" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Daily_Activity" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Daily_Time_24h_Check" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Plate_DestDay" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Surcharge_50pct_1Trip" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Manual_Extra_Trips" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Manual_Return_Trips" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="NoWork_Outbound_50pct" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Phantom_Trip_Candidates" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Hints_DoubleOrigin" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer_Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer_Trips_Per_Day" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit_Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trip_Detail" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trips_Pricing_All" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unmatched_Log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Activity" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Time_24h_Check" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plate_DestDay" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Surcharge_50pct_1Trip" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Extra_Trips" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Return_Trips" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoWork_Outbound_50pct" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phantom_Trip_Candidates" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hints_DoubleOrigin" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customer_Summary'!$A$1:$C$8</definedName>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05 20:19</t>
+          <t>2026-05-08 15:11</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-04-12–2026-04-15=8,000 / ปกติ=7,500</t>
+          <t>2026-05-01–2026-05-31=6,500 @31.00-31.99, step 1.50%/฿ / 2026-04-12–2026-04-15=8,000 @50.00-50.99, step 1.50%/฿, floor 6,500 / 2026-04-01–2026-04-30=7,500 @50.00-50.99, step 1.50%/฿, floor 6,500 / ปกติ=7,500 @50.00-50.99, step 1.50%/฿</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>811000</v>
+        <v>808500</v>
       </c>
     </row>
     <row r="14">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>7500</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="16">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>164500</v>
+        <v>163500</v>
       </c>
     </row>
     <row r="21">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1013000</v>
+        <v>1005750</v>
       </c>
     </row>
   </sheetData>
@@ -2837,10 +2837,10 @@
         <v>3750</v>
       </c>
       <c r="H61" s="7" t="n">
-        <v>7500</v>
+        <v>0</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>26250</v>
+        <v>18750</v>
       </c>
     </row>
     <row r="62">
@@ -3323,19 +3323,19 @@
         <v>1</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F76" s="6" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G76" s="6" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H76" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I76" s="6" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="77">
@@ -3356,19 +3356,19 @@
         <v>1</v>
       </c>
       <c r="E77" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F77" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G77" s="7" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H77" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I77" s="7" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
     </row>
   </sheetData>
@@ -4968,10 +4968,10 @@
       </c>
       <c r="J37" s="2" t="inlineStr"/>
       <c r="K37" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="L37" s="7" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
     </row>
     <row r="38">
@@ -5010,10 +5010,10 @@
       </c>
       <c r="J38" s="5" t="inlineStr"/>
       <c r="K38" s="6" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
     </row>
     <row r="39">
@@ -5245,7 +5245,7 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="41" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5280,11 +5280,11 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>7500</v>
+        <v>3750</v>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>ค่าขนส่งงานขากลับ (manual — ไม่มีใน GPS)</t>
+          <t>ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก</t>
         </is>
       </c>
     </row>
@@ -5777,7 +5777,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>811000</v>
+        <v>808500</v>
       </c>
     </row>
     <row r="3">
@@ -5807,7 +5807,7 @@
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>7500</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="5">
@@ -5837,7 +5837,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>164500</v>
+        <v>163500</v>
       </c>
     </row>
     <row r="7">
@@ -5867,7 +5867,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1013000</v>
+        <v>1005750</v>
       </c>
     </row>
   </sheetData>
@@ -8323,14 +8323,14 @@
         <v>3750</v>
       </c>
       <c r="H57" s="7" t="n">
-        <v>7500</v>
+        <v>3750</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>26250</v>
+        <v>22500</v>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว) | เที่ยวเพิ่ม (ไม่มีใน GPS): P&amp;G → Oatside (เที่ยวเพิ่ม — ไม่มีใน GPS) (+7,500฿) | ขากลับ (manual): ค่าขนส่งงานขากลับ (manual — ไม่มีใน GPS) (+7,500฿)</t>
+          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว) | เที่ยวเพิ่ม (ไม่มีใน GPS): P&amp;G → Oatside (เที่ยวเพิ่ม — ไม่มีใน GPS) (+7,500฿) | ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,750฿)</t>
         </is>
       </c>
     </row>
@@ -8770,19 +8770,19 @@
         <v>1</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F69" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G69" s="7" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H69" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
@@ -8808,19 +8808,19 @@
         <v>1</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="F70" s="6" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="G70" s="6" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="H70" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I70" s="6" t="n">
-        <v>11250</v>
+        <v>9750</v>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
@@ -10312,7 +10312,7 @@
         <v>1</v>
       </c>
       <c r="V16" s="6" t="n">
-        <v>8000</v>
+        <v>7500</v>
       </c>
       <c r="W16" s="6" t="n">
         <v>4000</v>
@@ -10488,7 +10488,7 @@
         <v>1</v>
       </c>
       <c r="V18" s="6" t="n">
-        <v>8000</v>
+        <v>7500</v>
       </c>
       <c r="W18" s="6" t="n">
         <v>0</v>
@@ -10576,7 +10576,7 @@
         <v>1</v>
       </c>
       <c r="V19" s="7" t="n">
-        <v>8000</v>
+        <v>7500</v>
       </c>
       <c r="W19" s="7" t="n">
         <v>4000</v>
@@ -10664,7 +10664,7 @@
         <v>1</v>
       </c>
       <c r="V20" s="6" t="n">
-        <v>8000</v>
+        <v>7500</v>
       </c>
       <c r="W20" s="6" t="n">
         <v>4000</v>
@@ -13132,7 +13132,7 @@
         <v>1</v>
       </c>
       <c r="V48" s="6" t="n">
-        <v>7500</v>
+        <v>8000</v>
       </c>
       <c r="W48" s="6" t="n">
         <v>0</v>
@@ -13312,7 +13312,7 @@
         <v>1</v>
       </c>
       <c r="V50" s="6" t="n">
-        <v>7500</v>
+        <v>8000</v>
       </c>
       <c r="W50" s="6" t="n">
         <v>3750</v>
@@ -13488,7 +13488,7 @@
         <v>1</v>
       </c>
       <c r="V52" s="6" t="n">
-        <v>7500</v>
+        <v>8000</v>
       </c>
       <c r="W52" s="6" t="n">
         <v>3750</v>
@@ -16776,7 +16776,7 @@
         <v>0</v>
       </c>
       <c r="Z89" s="7" t="n">
-        <v>7500</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="90">
@@ -18176,10 +18176,10 @@
         <v>1</v>
       </c>
       <c r="V105" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="W105" s="7" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="X105" s="7" t="n">
         <v>0</v>
@@ -18264,10 +18264,10 @@
         <v>1</v>
       </c>
       <c r="V106" s="6" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="W106" s="6" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="X106" s="6" t="n">
         <v>0</v>
@@ -18700,7 +18700,7 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>8000</v>
+        <v>7500</v>
       </c>
       <c r="D16" s="6" t="n">
         <v>4000</v>
@@ -18750,7 +18750,7 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>8000</v>
+        <v>7500</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>0</v>
@@ -18775,7 +18775,7 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>8000</v>
+        <v>7500</v>
       </c>
       <c r="D19" s="7" t="n">
         <v>4000</v>
@@ -18800,7 +18800,7 @@
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>8000</v>
+        <v>7500</v>
       </c>
       <c r="D20" s="6" t="n">
         <v>4000</v>
@@ -19500,7 +19500,7 @@
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>7500</v>
+        <v>8000</v>
       </c>
       <c r="D48" s="6" t="n">
         <v>0</v>
@@ -19550,7 +19550,7 @@
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>7500</v>
+        <v>8000</v>
       </c>
       <c r="D50" s="6" t="n">
         <v>3750</v>
@@ -19600,7 +19600,7 @@
         </is>
       </c>
       <c r="C52" s="6" t="n">
-        <v>7500</v>
+        <v>8000</v>
       </c>
       <c r="D52" s="6" t="n">
         <v>3750</v>
@@ -20537,7 +20537,7 @@
         <v>0</v>
       </c>
       <c r="G89" s="7" t="n">
-        <v>7500</v>
+        <v>3750</v>
       </c>
     </row>
     <row r="90">
@@ -20925,10 +20925,10 @@
         </is>
       </c>
       <c r="C105" s="7" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="D105" s="7" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="E105" s="7" t="n">
         <v>0</v>
@@ -20950,10 +20950,10 @@
         </is>
       </c>
       <c r="C106" s="6" t="n">
-        <v>7500</v>
+        <v>6500</v>
       </c>
       <c r="D106" s="6" t="n">
-        <v>3750</v>
+        <v>3250</v>
       </c>
       <c r="E106" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix oatside 100% downtime column mapping
Prevent +100% surcharge from silently landing in the wrong bucket by adding an explicit +50/+100 regression guard and clearer pricing export headers, then rebuild and redeploy the Oatside report with verified daily-diesel step pricing.
</commit_message>
<xml_diff>
--- a/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
+++ b/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08 15:56</t>
+          <t>2026-05-08 16:35</t>
         </is>
       </c>
     </row>
@@ -18297,9 +18297,9 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -18321,17 +18321,17 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Downtime_0_trip_baht</t>
+          <t>Downtime_50_baht</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Downtime_1_trip_baht</t>
+          <t>Downtime_100_baht</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Blank_run_baht</t>
+          <t>Blank_run_50_baht</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">

</xml_diff>

<commit_message>
﻿Standardize Oatside monetary output to 2 decimal places.
Keep calculation precision unchanged and apply 2dp formatting only at report presentation/export layers across HTML, XLSX, and new CSV table exports, then rebuild and deploy publish output.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
+++ b/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
@@ -135,10 +135,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08 16:35</t>
+          <t>2026-05-08 17:39</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01–2026-05-31=6,500 @31.00-31.99, step 1.50%/฿ / 2026-04-12–2026-04-15=8,000 @50.00-50.99, step 1.50%/฿, floor 6,500 / 2026-04-01–2026-04-30=7,500 @50.00-50.99, step 1.50%/฿, floor 6,500 / ปกติ=7,500 @50.00-50.99, step 1.50%/฿</t>
+          <t>2026-05-01–2026-05-31=6,500.00 @31.00-31.99, step 1.50%/฿ / 2026-04-12–2026-04-15=8,000.00 @50.00-50.99, step 1.50%/฿, floor 6,500.00 / 2026-04-01–2026-04-30=7,500.00 @50.00-50.99, step 1.50%/฿, floor 6,500.00 / ปกติ=7,500.00 @50.00-50.99, step 1.50%/฿</t>
         </is>
       </c>
     </row>
@@ -8330,7 +8330,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว) | เที่ยวเพิ่ม (ไม่มีใน GPS): P&amp;G → Oatside (เที่ยวเพิ่ม — ไม่มีใน GPS) (+7,500฿) | ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,250฿)</t>
+          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว) | เที่ยวเพิ่ม (ไม่มีใน GPS): P&amp;G → Oatside (เที่ยวเพิ่ม — ไม่มีใน GPS) (+7,500.00฿) | ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,250.00฿)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Oatside: cut May trips from report output window
Add configurable report date window and set report_end_date to 2026-04-30 so May data is excluded from Oatside report generation and published artifacts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
+++ b/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
@@ -26,19 +26,19 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customer_Summary'!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Customer_Trips_Per_Day'!$A$1:$C$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit_Log'!$A$1:$J$70</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$106</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Trips_Pricing_All'!$A$1:$G$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Customer_Trips_Per_Day'!$A$1:$C$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit_Log'!$A$1:$J$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Trips_Pricing_All'!$A$1:$G$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Unmatched_Log'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Daily_Activity'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$73</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$77</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Daily_Activity'!$A$1:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Phantom_Trip_Candidates'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Phantom_Trip_Candidates'!$A$1:$E$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Hints_DoubleOrigin'!$A$1:$D$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08 18:09</t>
+          <t>2026-05-08 18:39</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>735782.46</v>
+        <v>720918.4</v>
       </c>
     </row>
     <row r="14">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>147751</v>
+        <v>140319</v>
       </c>
     </row>
     <row r="21">
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>912806</v>
+        <v>890510</v>
       </c>
     </row>
   </sheetData>
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3305,74 +3305,8 @@
         <v>9750</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>71-5042</t>
-        </is>
-      </c>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>BigC</t>
-        </is>
-      </c>
-      <c r="D76" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E76" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="F76" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="G76" s="6" t="n">
-        <v>3716</v>
-      </c>
-      <c r="H76" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I76" s="6" t="n">
-        <v>11148.03</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E77" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="F77" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="G77" s="7" t="n">
-        <v>3716</v>
-      </c>
-      <c r="H77" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I77" s="7" t="n">
-        <v>11148.03</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I77"/>
+  <autoFilter ref="A1:I75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3383,7 +3317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4934,21 +4868,21 @@
     </row>
     <row r="37">
       <c r="A37" s="9" t="n">
-        <v>46143</v>
+        <v>46133</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-6802</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>downtime_origin_day</t>
+          <t>midnight_full</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
@@ -4956,31 +4890,39 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (20.96h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
+        </is>
+      </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr"/>
+          <t>2026-04-21 16:38:59</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-22 13:36:47</t>
+        </is>
+      </c>
       <c r="K37" s="7" t="n">
-        <v>7432.03</v>
+        <v>6645.86</v>
       </c>
       <c r="L37" s="7" t="n">
-        <v>3716</v>
+        <v>6645</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
-        <v>46143</v>
+        <v>46133</v>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8681</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -4990,7 +4932,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>downtime_origin_day</t>
+          <t>midnight_full</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
@@ -4998,22 +4940,30 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
-      <c r="H38" s="5" t="inlineStr"/>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (21.30h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
+        </is>
+      </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="J38" s="5" t="inlineStr"/>
+          <t>2026-04-21 13:37:02</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:55:11</t>
+        </is>
+      </c>
       <c r="K38" s="6" t="n">
-        <v>7432.03</v>
+        <v>6645.86</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>3716</v>
+        <v>6645</v>
       </c>
     </row>
     <row r="39">
@@ -5022,7 +4972,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>71-6802</t>
+          <t>71-9629</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -5046,17 +4996,17 @@
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (20.96h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
+          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (18.79h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 16:38:59</t>
+          <t>2026-04-21 09:15:51</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22 13:36:47</t>
+          <t>2026-04-22 04:03:28</t>
         </is>
       </c>
       <c r="K39" s="7" t="n">
@@ -5066,108 +5016,8 @@
         <v>6645</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="n">
-        <v>46133</v>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>71-8681</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>midnight_full</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr"/>
-      <c r="H40" s="5" t="inlineStr">
-        <is>
-          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (21.30h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
-        </is>
-      </c>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-21 13:37:02</t>
-        </is>
-      </c>
-      <c r="J40" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-22 10:55:11</t>
-        </is>
-      </c>
-      <c r="K40" s="6" t="n">
-        <v>6645.86</v>
-      </c>
-      <c r="L40" s="6" t="n">
-        <v>6645</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="n">
-        <v>46133</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>71-9629</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>midnight_full</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (18.79h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-21 09:15:51</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-22 04:03:28</t>
-        </is>
-      </c>
-      <c r="K41" s="7" t="n">
-        <v>6645.86</v>
-      </c>
-      <c r="L41" s="7" t="n">
-        <v>6645</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L41"/>
+  <autoFilter ref="A1:L39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5609,7 +5459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5667,8 +5517,50 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>71-5042</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>46143</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>7432.03</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>No matched trip on this trip_date; OAT rule: charge 1 full trip (review before adding to grand total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>72-1217</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>46143</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>7432.03</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>No matched trip on this trip_date; OAT rule: charge 1 full trip (review before adding to grand total)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E2"/>
+  <autoFilter ref="A1:E4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5777,7 +5669,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>735782.46</v>
+        <v>720918.4</v>
       </c>
     </row>
     <row r="3">
@@ -5837,7 +5729,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>147751</v>
+        <v>140319</v>
       </c>
     </row>
     <row r="7">
@@ -5867,7 +5759,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>912806</v>
+        <v>890510</v>
       </c>
     </row>
   </sheetData>
@@ -5882,7 +5774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6116,19 +6008,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C21"/>
+  <autoFilter ref="A1:C20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6139,7 +6020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8752,84 +8633,8 @@
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>71-5042</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>BigC</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E69" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="F69" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="G69" s="7" t="n">
-        <v>3716</v>
-      </c>
-      <c r="H69" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I69" s="7" t="n">
-        <v>11148.03</v>
-      </c>
-      <c r="J69" s="2" t="inlineStr">
-        <is>
-          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว)</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E70" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="F70" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="G70" s="6" t="n">
-        <v>3716</v>
-      </c>
-      <c r="H70" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I70" s="6" t="n">
-        <v>11148.03</v>
-      </c>
-      <c r="J70" s="5" t="inlineStr">
-        <is>
-          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J70"/>
+  <autoFilter ref="A1:J68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8840,7 +8645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z106"/>
+  <dimension ref="A1:Z104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18103,184 +17908,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B105" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="C105" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>BigC</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>71-5042</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr">
-        <is>
-          <t>71-5042 ณัชพน หัวลาก10W</t>
-        </is>
-      </c>
-      <c r="G105" s="2" t="inlineStr">
-        <is>
-          <t>13.8</t>
-        </is>
-      </c>
-      <c r="H105" s="2" t="inlineStr">
-        <is>
-          <t>14.9</t>
-        </is>
-      </c>
-      <c r="I105" s="11" t="n">
-        <v>46143.26266203704</v>
-      </c>
-      <c r="J105" s="11" t="n">
-        <v>46143.48762731482</v>
-      </c>
-      <c r="K105" s="2" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="L105" s="11" t="n">
-        <v>46143.56759259259</v>
-      </c>
-      <c r="M105" s="11" t="n">
-        <v>46143.6196875</v>
-      </c>
-      <c r="N105" s="2" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="O105" s="2" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="P105" s="2" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="Q105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R105" s="2" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="S105" s="2" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="T105" s="2" t="n"/>
-      <c r="U105" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="V105" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="W105" s="7" t="n">
-        <v>3716</v>
-      </c>
-      <c r="X105" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y105" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z105" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B106" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="C106" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D106" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="E106" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="F106" s="5" t="inlineStr">
-        <is>
-          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
-        </is>
-      </c>
-      <c r="G106" s="5" t="inlineStr">
-        <is>
-          <t>7.14</t>
-        </is>
-      </c>
-      <c r="H106" s="5" t="inlineStr">
-        <is>
-          <t>7.14</t>
-        </is>
-      </c>
-      <c r="I106" s="10" t="n">
-        <v>46143.82527777777</v>
-      </c>
-      <c r="J106" s="10" t="n">
-        <v>46143.89219907407</v>
-      </c>
-      <c r="K106" s="5" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="L106" s="10" t="n">
-        <v>46143.96318287037</v>
-      </c>
-      <c r="M106" s="10" t="n">
-        <v>46143.97673611111</v>
-      </c>
-      <c r="N106" s="5" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="O106" s="5" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="P106" s="5" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="Q106" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R106" s="5" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="S106" s="5" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="T106" s="5" t="n"/>
-      <c r="U106" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="V106" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="W106" s="6" t="n">
-        <v>3716</v>
-      </c>
-      <c r="X106" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y106" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z106" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Z106"/>
+  <autoFilter ref="A1:Z104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18291,7 +17920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G106"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20915,58 +20544,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B105" s="2" t="inlineStr">
-        <is>
-          <t>71-5042</t>
-        </is>
-      </c>
-      <c r="C105" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="D105" s="7" t="n">
-        <v>3716</v>
-      </c>
-      <c r="E105" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F105" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G105" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B106" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="D106" s="6" t="n">
-        <v>3716</v>
-      </c>
-      <c r="E106" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F106" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G106" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G106"/>
+  <autoFilter ref="A1:G104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21524,7 +21103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22136,37 +21715,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
+  <autoFilter ref="A1:I20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22177,7 +21727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M73"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -25552,102 +25102,8 @@
         <v>15.4</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>71-5042</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>BigC</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="E72" s="5" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="F72" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="G72" s="5" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="H72" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I72" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J72" s="5" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="K72" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="L72" s="5" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="M72" s="5" t="n">
-        <v>15.43</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="E73" s="2" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="F73" s="2" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="G73" s="2" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J73" s="2" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="K73" s="2" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="L73" s="2" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="M73" s="2" t="n">
-        <v>20.37</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M73"/>
+  <autoFilter ref="A1:M71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
backup: auto save before claude
</commit_message>
<xml_diff>
--- a/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
+++ b/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
@@ -25,7 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hints_DoubleOrigin" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customer_Summary'!$A$1:$C$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customer_Summary'!$A$1:$C$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Customer_Trips_Per_Day'!$A$1:$C$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit_Log'!$A$1:$J$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$104</definedName>
@@ -35,7 +35,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Phantom_Trip_Candidates'!$A$1:$E$4</definedName>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08 18:39</t>
+          <t>2026-05-09 00:22</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>720918.4</v>
+        <v>713418.4</v>
       </c>
     </row>
     <row r="14">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>7500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>890510</v>
+        <v>883010</v>
       </c>
     </row>
   </sheetData>
@@ -2825,13 +2825,13 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E61" s="7" t="n">
         <v>6546.17</v>
       </c>
       <c r="F61" s="7" t="n">
-        <v>14046</v>
+        <v>6546.17</v>
       </c>
       <c r="G61" s="7" t="n">
         <v>3273</v>
@@ -2840,7 +2840,7 @@
         <v>0</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>17319</v>
+        <v>9819</v>
       </c>
     </row>
     <row r="62">
@@ -5028,13 +5028,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5059,26 +5059,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="n">
-        <v>46134</v>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="n">
-        <v>7500</v>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>P&amp;G → Oatside (เที่ยวเพิ่ม — ไม่มีใน GPS)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D2"/>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5632,7 +5614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5669,101 +5651,86 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>720918.4</v>
+        <v>713418.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>R</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ในนั้น: เที่ยวเพิ่ม (manual_extra_trips ไม่มีใน GPS)</t>
+          <t>ค่าขนส่งขากลับ (manual_return_trips — ไม่เพิ่มจำนวน matched)</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>7500</v>
+        <v>3273.09</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>ค่าขนส่งขากลับ (manual_return_trips — ไม่เพิ่มจำนวน matched)</t>
+          <t>ค่าชดเชยเที่ยวขาด (min 2/คัน/วัน) — ไม่เก็บเงิน (ใช้ชาร์จ 50% วันละ 1 เที่ยวแทน)</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>3273.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ค่าชดเชยเที่ยวขาด (min 2/คัน/วัน) — ไม่เก็บเงิน (ใช้ชาร์จ 50% วันละ 1 เที่ยวแทน)</t>
+          <t>ชาร์จ 50% วันที่วิ่งได้ 1 เที่ยว (หลัง override)</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>0</v>
+        <v>140319</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>ชาร์จ 50% วันที่วิ่งได้ 1 เที่ยว (หลัง override)</t>
+          <t>No-work recovery outbound 50pct (first matched trip that Dest_In day on recovery dates)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>140319</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>No-work recovery outbound 50pct (first matched trip that Dest_In day on recovery dates)</t>
+          <t>Grand (A+C+D+R)</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>26000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Grand (A+C+D+R)</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>890510</v>
+        <v>883010</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C8"/>
+  <autoFilter ref="A1:C7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5947,7 +5914,7 @@
         <v>46134</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>4</v>
@@ -8192,13 +8159,13 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E57" s="7" t="n">
         <v>6546.17</v>
       </c>
       <c r="F57" s="7" t="n">
-        <v>14046</v>
+        <v>6546.17</v>
       </c>
       <c r="G57" s="7" t="n">
         <v>3273</v>
@@ -8207,11 +8174,11 @@
         <v>3273</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>20592</v>
+        <v>13092</v>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว) | เที่ยวเพิ่ม (ไม่มีใน GPS): P&amp;G → Oatside (เที่ยวเพิ่ม — ไม่มีใน GPS) (+7,500.00฿) | ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,273.09฿)</t>
+          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว) | ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,273.09฿)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Oatside trips display: attach no-finish-day 100% to next trip's row
- _split_fifty_surcharge_50_100 now buckets no_finish_day / one_trip_billed_day correctly
- attach_no_finish_to_next_trip re-keys no-finish surcharges to the next trip's billed_day per plate
- Trips page now shows +100% column populated on the first trip after a no-finish day
- _assert_pricing_bucket_mapping updated to use same attachment for consistency
- Example: 71-5041 row Origin 5/7→Dest_Out 5/8 now shows ค่าขนส่ง 7,168 + เสียเวลา+50% 3,584 + เสียเวลา+100% 7,264

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
+++ b/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05 21:22</t>
+          <t>2026-06-05 22:49</t>
         </is>
       </c>
     </row>
@@ -14427,7 +14427,7 @@
         <v>3632</v>
       </c>
       <c r="X3" s="7" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="Y3" s="7" t="n">
         <v>0</v>
@@ -14515,7 +14515,7 @@
         <v>3632</v>
       </c>
       <c r="X4" s="6" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="Y4" s="6" t="n">
         <v>0</v>
@@ -14603,7 +14603,7 @@
         <v>3632</v>
       </c>
       <c r="X5" s="7" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="Y5" s="7" t="n">
         <v>0</v>
@@ -14691,7 +14691,7 @@
         <v>3632</v>
       </c>
       <c r="X6" s="6" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="Y6" s="6" t="n">
         <v>0</v>
@@ -15747,7 +15747,7 @@
         <v>3584</v>
       </c>
       <c r="X18" s="6" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="Y18" s="6" t="n">
         <v>0</v>
@@ -20591,7 +20591,7 @@
         <v>3680</v>
       </c>
       <c r="X73" s="7" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="Y73" s="7" t="n">
         <v>0</v>
@@ -25171,7 +25171,7 @@
         <v>3680</v>
       </c>
       <c r="X125" s="7" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="Y125" s="7" t="n">
         <v>0</v>
@@ -25347,7 +25347,7 @@
         <v>3680</v>
       </c>
       <c r="X127" s="7" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="Y127" s="7" t="n">
         <v>0</v>
@@ -25523,7 +25523,7 @@
         <v>3680</v>
       </c>
       <c r="X129" s="7" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="Y129" s="7" t="n">
         <v>0</v>
@@ -27930,7 +27930,7 @@
         <v>3632</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="F3" s="7" t="n">
         <v>0</v>
@@ -27955,7 +27955,7 @@
         <v>3632</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="F4" s="6" t="n">
         <v>0</v>
@@ -27980,7 +27980,7 @@
         <v>3632</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>0</v>
@@ -28005,7 +28005,7 @@
         <v>3632</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>0</v>
@@ -28305,7 +28305,7 @@
         <v>3584</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>0</v>
+        <v>7264</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>0</v>
@@ -29680,7 +29680,7 @@
         <v>3680</v>
       </c>
       <c r="E73" s="7" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="F73" s="7" t="n">
         <v>0</v>
@@ -30980,7 +30980,7 @@
         <v>3680</v>
       </c>
       <c r="E125" s="7" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="F125" s="7" t="n">
         <v>0</v>
@@ -31030,7 +31030,7 @@
         <v>3680</v>
       </c>
       <c r="E127" s="7" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="F127" s="7" t="n">
         <v>0</v>
@@ -31080,7 +31080,7 @@
         <v>3680</v>
       </c>
       <c r="E129" s="7" t="n">
-        <v>0</v>
+        <v>7360</v>
       </c>
       <c r="F129" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Oatside พ.ค.: add backhaul/deadhead 50% (+29,440) + daily↔GPS recon
- manual_return_trips: 8 BH/ตีเปล่า entries from keyed daily that GPS can't see
  (5042 01/05; 8009 10,11,20,22; 8002 20; 8001 20,21) = +29,440 บาท
- use explicit amount_baht (avoids percent-entry +0฿ render bug on matched days)
- 8001/8005 20/05: net only the leg base doesn't already bill — base_trips_revenue_baht
  charges every matched movement full-rate (empty runs incl.), so avoid double-count
- decisions: #1 no_finish keeps waiting-day rate (correct, not a bug);
  #3 demurrage system>=keyer for all plates -> no override added
- RECON_STATE.md: full reconciliation record; _recon/_xl/_apply scripts as audit trail
- regenerated oatside-apr2026 report set (per-day badges now reconcile with grand)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
+++ b/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
@@ -36,7 +36,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$125</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Phantom_Trip_Candidates'!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Hints_DoubleOrigin'!$A$1:$D$1</definedName>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05 22:49</t>
+          <t>2026-06-08 18:37</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>3250</v>
+        <v>32690</v>
       </c>
     </row>
     <row r="16">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1469970</v>
+        <v>1499410</v>
       </c>
     </row>
   </sheetData>
@@ -923,10 +923,10 @@
         <v>3632</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="4">
@@ -1946,10 +1946,10 @@
         <v>3584</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>10752</v>
+        <v>14336</v>
       </c>
     </row>
     <row r="35">
@@ -2045,10 +2045,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>14336</v>
+        <v>17920</v>
       </c>
     </row>
     <row r="38">
@@ -3068,10 +3068,10 @@
         <v>3728</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I68" s="6" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="69">
@@ -3101,10 +3101,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
     </row>
     <row r="70">
@@ -3167,10 +3167,10 @@
         <v>3728</v>
       </c>
       <c r="H71" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="72">
@@ -3233,10 +3233,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
     </row>
     <row r="74">
@@ -3497,10 +3497,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
     </row>
     <row r="82">
@@ -8587,13 +8587,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="41" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8636,8 +8636,152 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="9" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>71-5042</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>3632</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ตีเปล่าไป P&amp;G 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>71-8002</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>3728</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>3728</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>71-8001</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>3728</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>BH ขากลับเพิ่ม 50% (base คิด ตีเปล่า+BH#1 = 1 เที่ยวแล้ว)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>71-8001</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>3728</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>3728</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D2"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8853,7 +8997,7 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>3250</v>
+        <v>32690</v>
       </c>
     </row>
     <row r="4">
@@ -8913,7 +9057,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1469970</v>
+        <v>1499410</v>
       </c>
     </row>
   </sheetData>
@@ -9438,14 +9582,14 @@
         <v>3632</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว)</t>
+          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว) | ขากลับ (manual): ตีเปล่าไป P&amp;G 50% (+3,632.00฿)</t>
         </is>
       </c>
     </row>
@@ -10616,14 +10760,14 @@
         <v>3584</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>10752</v>
+        <v>14336</v>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว)</t>
+          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,584.00฿)</t>
         </is>
       </c>
     </row>
@@ -10730,14 +10874,14 @@
         <v>0</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>14336</v>
+        <v>17920</v>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว)</t>
+          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,584.00฿)</t>
         </is>
       </c>
     </row>
@@ -11908,14 +12052,14 @@
         <v>3728</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I68" s="6" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว)</t>
+          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว) | ขากลับ (manual): BH ขากลับเพิ่ม 50% (base คิด ตีเปล่า+BH#1 = 1 เที่ยวแล้ว) (+3,728.00฿)</t>
         </is>
       </c>
     </row>
@@ -11946,14 +12090,14 @@
         <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว)</t>
+          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,728.00฿)</t>
         </is>
       </c>
     </row>
@@ -12022,14 +12166,14 @@
         <v>3728</v>
       </c>
       <c r="H71" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว)</t>
+          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,728.00฿)</t>
         </is>
       </c>
     </row>
@@ -12098,14 +12242,14 @@
         <v>0</v>
       </c>
       <c r="H73" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว)</t>
+          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,728.00฿)</t>
         </is>
       </c>
     </row>
@@ -12402,14 +12546,14 @@
         <v>0</v>
       </c>
       <c r="H81" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว)</t>
+          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,728.00฿)</t>
         </is>
       </c>
     </row>
@@ -14345,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="Z2" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
     </row>
     <row r="3">
@@ -17249,7 +17393,7 @@
         <v>0</v>
       </c>
       <c r="Z35" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
     </row>
     <row r="36">
@@ -17601,7 +17745,7 @@
         <v>0</v>
       </c>
       <c r="Z39" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
     </row>
     <row r="40">
@@ -21477,7 +21621,7 @@
         <v>0</v>
       </c>
       <c r="Z83" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="84">
@@ -21565,7 +21709,7 @@
         <v>0</v>
       </c>
       <c r="Z84" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="85">
@@ -21917,7 +22061,7 @@
         <v>0</v>
       </c>
       <c r="Z88" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="89">
@@ -22093,7 +22237,7 @@
         <v>0</v>
       </c>
       <c r="Z90" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="91">
@@ -22885,7 +23029,7 @@
         <v>0</v>
       </c>
       <c r="Z99" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="100">
@@ -27911,7 +28055,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
     </row>
     <row r="3">
@@ -28736,7 +28880,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
     </row>
     <row r="36">
@@ -28836,7 +28980,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
     </row>
     <row r="40">
@@ -29936,7 +30080,7 @@
         <v>0</v>
       </c>
       <c r="G83" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="84">
@@ -29961,7 +30105,7 @@
         <v>0</v>
       </c>
       <c r="G84" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="85">
@@ -30061,7 +30205,7 @@
         <v>0</v>
       </c>
       <c r="G88" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="89">
@@ -30111,7 +30255,7 @@
         <v>0</v>
       </c>
       <c r="G90" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="91">
@@ -30336,7 +30480,7 @@
         <v>0</v>
       </c>
       <c r="G99" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="100">

</xml_diff>

<commit_message>
Oatside: fix manual_return +0฿ render for percent-based entries
merge_manual_return_into_pday (existing-row) and merge_manual_return_into_audit
(not-hit + no-note paths) used m.amount_baht (=0 for percent_of_trip_rate entries)
instead of manual_return_amount_baht(m, cfg). Per-day/audit showed "+0.00฿" while
the grand total counted the 50% correctly. Both now use the computed amount.

Verified: 72-1217 (April, percent 50) renders +3,250฿; zero "+0.00฿" remaining.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
+++ b/Oatside/Oatside_PG_Trip_Summary_By_Site.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08 18:37</t>
+          <t>2026-06-08 18:47</t>
         </is>
       </c>
     </row>
@@ -9544,14 +9544,14 @@
         <v>0</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>0</v>
+        <v>3250</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>0</v>
+        <v>3250</v>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+0.00฿)</t>
+          <t>ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,250.00฿)</t>
         </is>
       </c>
     </row>

</xml_diff>